<commit_message>
feat: add bolt group generation and slim docs workflow
Add Bolt_Group template/validation/output support and move Item_Code ordering fully to project_config item_order (including G,B) without hardcoded sort exceptions. Slim project documentation by replacing progress tracking with changelog/rules-based guidance and include new harness case inputs/expected outputs for regression alignment.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/data/Item_Code_DB.xlsx
+++ b/data/Item_Code_DB.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -988,6 +988,28 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>BOLT&amp;NUT</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>BOLT</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Bolt_Group</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: simplify project baseline and consolidate core rules
Reduce repository surface by removing non-essential docs/rules/assets, consolidate project policy into core rule files, and keep generator/data aligned with the updated baseline.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/data/Item_Code_DB.xlsx
+++ b/data/Item_Code_DB.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1010,6 +1010,160 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>GATE VALVE</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>GATE VALVE</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Valve_Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>VB</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>GLOBE VALVE</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>GLOBE VALVE</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Valve_Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>VC</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>CHECK VALVE</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>CHECK VALVE</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Valve_Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>VL</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>BALL VALVE</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>BALL VALVE</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Valve_Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>VU</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>BUTTERFLY VALVE</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>BUTTERFLY VALVE</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Valve_Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>VP</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>PLUG VALVE</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>PLUG VALVE</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Valve_Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>DIAPHRAGM VALVE</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>DIAPHRAGM VALVE</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Valve_Group</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>